<commit_message>
cleans metadata and summary doc
</commit_message>
<xml_diff>
--- a/data-raw/metadata/battle_redd_summary_metadata.xlsx
+++ b/data-raw/metadata/battle_redd_summary_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-battle-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26AEEFE3-9178-4AD2-801C-D26D69865A2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80FD6FEB-1D5D-4305-A569-57A020457C77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4220" yWindow="1960" windowWidth="17070" windowHeight="11490" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6680" yWindow="2150" windowWidth="16900" windowHeight="9990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
   <si>
     <t xml:space="preserve">attribute_name </t>
   </si>
@@ -140,6 +140,15 @@
   </si>
   <si>
     <t>Survey reach  where survey was done</t>
+  </si>
+  <si>
+    <t>Indicates if year should be added to analysis if TRUE</t>
+  </si>
+  <si>
+    <t>include_modeling</t>
+  </si>
+  <si>
+    <t>nominal</t>
   </si>
 </sst>
 </file>
@@ -719,11 +728,21 @@
       <c r="Z5" s="7"/>
     </row>
     <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="4"/>
+      <c r="A6" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>36</v>
+      </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>

</xml_diff>